<commit_message>
Fix en excel consolidado
</commit_message>
<xml_diff>
--- a/RESULTADOS_EXPERIMENTO_CONSOLIDADO.xlsx
+++ b/RESULTADOS_EXPERIMENTO_CONSOLIDADO.xlsx
@@ -516,7 +516,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.24 GB (Disponible: 2.42 GB)</t>
+          <t>15.24 GB (Disponible: 4.22 GB)</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
         <v>30</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>45000</v>
+        <v>1500</v>
       </c>
       <c r="E4" s="5" t="n">
         <v>0</v>
@@ -699,10 +699,10 @@
         <v>0</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.386494</v>
+        <v>0.204966</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.204966</v>
+        <v>0.111713</v>
       </c>
     </row>
     <row r="5">
@@ -729,7 +729,7 @@
         <v>5005.909967</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.198718</v>
+        <v>0.202429</v>
       </c>
       <c r="H5" s="6" t="n">
         <v>0.109563</v>
@@ -759,7 +759,7 @@
         <v>7268.047</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.203351</v>
+        <v>0.200773</v>
       </c>
       <c r="H6" s="6" t="n">
         <v>0.09177</v>
@@ -789,7 +789,7 @@
         <v>9399.156367</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.215228</v>
+        <v>0.215384</v>
       </c>
       <c r="H7" s="6" t="n">
         <v>0.114656</v>
@@ -819,7 +819,7 @@
         <v>17188.910967</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.201761</v>
+        <v>0.204515</v>
       </c>
       <c r="H8" s="6" t="n">
         <v>0.11617</v>
@@ -849,7 +849,7 @@
         <v>35231.956933</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.213328</v>
+        <v>0.214741</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>0.120281</v>
@@ -962,10 +962,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.1234259</v>
+        <v>0.2000608</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>0.1234259</v>
+        <v>0.2000608</v>
       </c>
     </row>
     <row r="5">
@@ -993,10 +993,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.2381442</v>
+        <v>0.1234259</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>0.2381442</v>
+        <v>0.1234259</v>
       </c>
     </row>
     <row r="6">
@@ -1024,10 +1024,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.2832955</v>
+        <v>0.2381442</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>0.2832955</v>
+        <v>0.2381442</v>
       </c>
     </row>
     <row r="7">
@@ -1055,10 +1055,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.2615152</v>
+        <v>0.2832955</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>0.2615152</v>
+        <v>0.2832955</v>
       </c>
     </row>
     <row r="8">
@@ -1086,10 +1086,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.1117133</v>
+        <v>0.2615152</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>0.1117133</v>
+        <v>0.2615152</v>
       </c>
     </row>
     <row r="9">
@@ -1117,10 +1117,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.2166446</v>
+        <v>0.1117133</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>0.2166446</v>
+        <v>0.1117133</v>
       </c>
     </row>
     <row r="10">
@@ -1148,10 +1148,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.2389833</v>
+        <v>0.2166446</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>0.2389833</v>
+        <v>0.2166446</v>
       </c>
     </row>
     <row r="11">
@@ -1179,10 +1179,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0.2780455</v>
+        <v>0.2389833</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>0.2780455</v>
+        <v>0.2389833</v>
       </c>
     </row>
     <row r="12">
@@ -1210,10 +1210,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>0.2298738</v>
+        <v>0.2780455</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>0.2298738</v>
+        <v>0.2780455</v>
       </c>
     </row>
     <row r="13">
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>0.1468191</v>
+        <v>0.2298738</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>0.1468191</v>
+        <v>0.2298738</v>
       </c>
     </row>
     <row r="14">
@@ -1272,10 +1272,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>0.2788391</v>
+        <v>0.1468191</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>0.2788391</v>
+        <v>0.1468191</v>
       </c>
     </row>
     <row r="15">
@@ -1303,10 +1303,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>0.172061</v>
+        <v>0.2788391</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>0.172061</v>
+        <v>0.2788391</v>
       </c>
     </row>
     <row r="16">
@@ -1334,10 +1334,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>0.2247473</v>
+        <v>0.172061</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>0.2247473</v>
+        <v>0.172061</v>
       </c>
     </row>
     <row r="17">
@@ -1365,10 +1365,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>0.1229662</v>
+        <v>0.2247473</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>0.1229662</v>
+        <v>0.2247473</v>
       </c>
     </row>
     <row r="18">
@@ -1396,10 +1396,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>0.1220901</v>
+        <v>0.1229662</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>0.1220901</v>
+        <v>0.1229662</v>
       </c>
     </row>
     <row r="19">
@@ -1427,10 +1427,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>0.1854472</v>
+        <v>0.1220901</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>0.1854472</v>
+        <v>0.1220901</v>
       </c>
     </row>
     <row r="20">
@@ -1458,10 +1458,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>0.2379217</v>
+        <v>0.1854472</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>0.2379217</v>
+        <v>0.1854472</v>
       </c>
     </row>
     <row r="21">
@@ -1489,10 +1489,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>0.2208987</v>
+        <v>0.2379217</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>0.2208987</v>
+        <v>0.2379217</v>
       </c>
     </row>
     <row r="22">
@@ -1520,10 +1520,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>0.1285862</v>
+        <v>0.2208987</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>0.1285862</v>
+        <v>0.2208987</v>
       </c>
     </row>
     <row r="23">
@@ -1551,10 +1551,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>0.1955921</v>
+        <v>0.1285862</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>0.1955921</v>
+        <v>0.1285862</v>
       </c>
     </row>
     <row r="24">
@@ -1582,10 +1582,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>0.1940448</v>
+        <v>0.1955921</v>
       </c>
       <c r="I24" s="6" t="n">
-        <v>0.1940448</v>
+        <v>0.1955921</v>
       </c>
     </row>
     <row r="25">
@@ -1613,10 +1613,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>0.1832837</v>
+        <v>0.1940448</v>
       </c>
       <c r="I25" s="6" t="n">
-        <v>0.1832837</v>
+        <v>0.1940448</v>
       </c>
     </row>
     <row r="26">
@@ -1644,10 +1644,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>0.1752454</v>
+        <v>0.1832837</v>
       </c>
       <c r="I26" s="6" t="n">
-        <v>0.1752454</v>
+        <v>0.1832837</v>
       </c>
     </row>
     <row r="27">
@@ -1675,10 +1675,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>0.237883</v>
+        <v>0.1752454</v>
       </c>
       <c r="I27" s="6" t="n">
-        <v>0.237883</v>
+        <v>0.1752454</v>
       </c>
     </row>
     <row r="28">
@@ -1706,10 +1706,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>0.2736944</v>
+        <v>0.237883</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>0.2736944</v>
+        <v>0.237883</v>
       </c>
     </row>
     <row r="29">
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>0.2218911</v>
+        <v>0.2736944</v>
       </c>
       <c r="I29" s="6" t="n">
-        <v>0.2218911</v>
+        <v>0.2736944</v>
       </c>
     </row>
     <row r="30">
@@ -1768,10 +1768,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>0.1894443</v>
+        <v>0.2218911</v>
       </c>
       <c r="I30" s="6" t="n">
-        <v>0.1894443</v>
+        <v>0.2218911</v>
       </c>
     </row>
     <row r="31">
@@ -1799,10 +1799,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>0.237777</v>
+        <v>0.1894443</v>
       </c>
       <c r="I31" s="6" t="n">
-        <v>0.237777</v>
+        <v>0.1894443</v>
       </c>
     </row>
     <row r="32">
@@ -1830,10 +1830,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>0.2180408</v>
+        <v>0.237777</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>0.2180408</v>
+        <v>0.237777</v>
       </c>
     </row>
     <row r="33">
@@ -1861,10 +1861,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>0</v>
+        <v>0.2180408</v>
       </c>
       <c r="I33" s="6" t="n">
-        <v>0</v>
+        <v>0.2180408</v>
       </c>
     </row>
     <row r="34">
@@ -1886,16 +1886,16 @@
         <v>22.609</v>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0</v>
+        <v>2.23</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>0</v>
+        <v>0.037</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>0.1250019</v>
+        <v>0.3100512</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>0.1250019</v>
+        <v>0.3100512</v>
       </c>
     </row>
     <row r="35">
@@ -1917,16 +1917,16 @@
         <v>1450.047</v>
       </c>
       <c r="F35" s="5" t="n">
-        <v>0</v>
+        <v>20.36</v>
       </c>
       <c r="G35" s="5" t="n">
-        <v>0</v>
+        <v>1.23</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>0.1887559</v>
+        <v>0.1250019</v>
       </c>
       <c r="I35" s="6" t="n">
-        <v>0.1887559</v>
+        <v>0.1250019</v>
       </c>
     </row>
     <row r="36">
@@ -1948,16 +1948,16 @@
         <v>1450.375</v>
       </c>
       <c r="F36" s="5" t="n">
-        <v>0</v>
+        <v>13.16</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>0</v>
+        <v>0.785</v>
       </c>
       <c r="H36" s="6" t="n">
-        <v>0.2670515</v>
+        <v>0.1887559</v>
       </c>
       <c r="I36" s="6" t="n">
-        <v>0.2670515</v>
+        <v>0.1887559</v>
       </c>
     </row>
     <row r="37">
@@ -1979,16 +1979,16 @@
         <v>1454.688</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0</v>
+        <v>10.1</v>
       </c>
       <c r="G37" s="5" t="n">
-        <v>0</v>
+        <v>0.596</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>0.1987498</v>
+        <v>0.2670515</v>
       </c>
       <c r="I37" s="6" t="n">
-        <v>0.1987498</v>
+        <v>0.2670515</v>
       </c>
     </row>
     <row r="38">
@@ -2010,16 +2010,16 @@
         <v>1463.156</v>
       </c>
       <c r="F38" s="5" t="n">
-        <v>0</v>
+        <v>8.050000000000001</v>
       </c>
       <c r="G38" s="5" t="n">
-        <v>0</v>
+        <v>0.473</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>0.2364685</v>
+        <v>0.1987498</v>
       </c>
       <c r="I38" s="6" t="n">
-        <v>0.2364685</v>
+        <v>0.1987498</v>
       </c>
     </row>
     <row r="39">
@@ -2041,16 +2041,16 @@
         <v>1466.078</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>0</v>
+        <v>7.02</v>
       </c>
       <c r="G39" s="5" t="n">
-        <v>0</v>
+        <v>0.402</v>
       </c>
       <c r="H39" s="6" t="n">
-        <v>0.194044</v>
+        <v>0.2364685</v>
       </c>
       <c r="I39" s="6" t="n">
-        <v>0.194044</v>
+        <v>0.2364685</v>
       </c>
     </row>
     <row r="40">
@@ -2072,16 +2072,16 @@
         <v>2148.531</v>
       </c>
       <c r="F40" s="5" t="n">
-        <v>0</v>
+        <v>8.75</v>
       </c>
       <c r="G40" s="5" t="n">
-        <v>0</v>
+        <v>0.517</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>0.2688232</v>
+        <v>0.194044</v>
       </c>
       <c r="I40" s="6" t="n">
-        <v>0.2688232</v>
+        <v>0.194044</v>
       </c>
     </row>
     <row r="41">
@@ -2103,16 +2103,16 @@
         <v>2161.844</v>
       </c>
       <c r="F41" s="5" t="n">
-        <v>0</v>
+        <v>8.01</v>
       </c>
       <c r="G41" s="5" t="n">
-        <v>0</v>
+        <v>0.46</v>
       </c>
       <c r="H41" s="6" t="n">
-        <v>0.2447125</v>
+        <v>0.2688232</v>
       </c>
       <c r="I41" s="6" t="n">
-        <v>0.2447125</v>
+        <v>0.2688232</v>
       </c>
     </row>
     <row r="42">
@@ -2134,16 +2134,16 @@
         <v>2170.203</v>
       </c>
       <c r="F42" s="5" t="n">
-        <v>0</v>
+        <v>7.68</v>
       </c>
       <c r="G42" s="5" t="n">
-        <v>0</v>
+        <v>0.412</v>
       </c>
       <c r="H42" s="6" t="n">
-        <v>0.1250019</v>
+        <v>0.2447125</v>
       </c>
       <c r="I42" s="6" t="n">
-        <v>0.1250019</v>
+        <v>0.2447125</v>
       </c>
     </row>
     <row r="43">
@@ -2165,16 +2165,16 @@
         <v>2963.313</v>
       </c>
       <c r="F43" s="5" t="n">
-        <v>0</v>
+        <v>9.41</v>
       </c>
       <c r="G43" s="5" t="n">
-        <v>0</v>
+        <v>0.502</v>
       </c>
       <c r="H43" s="6" t="n">
-        <v>0.1625948</v>
+        <v>0.1250019</v>
       </c>
       <c r="I43" s="6" t="n">
-        <v>0.1625948</v>
+        <v>0.1250019</v>
       </c>
     </row>
     <row r="44">
@@ -2196,16 +2196,16 @@
         <v>2976.375</v>
       </c>
       <c r="F44" s="5" t="n">
-        <v>0</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>0</v>
+        <v>0.462</v>
       </c>
       <c r="H44" s="6" t="n">
-        <v>0.1095627</v>
+        <v>0.1625948</v>
       </c>
       <c r="I44" s="6" t="n">
-        <v>0.1095627</v>
+        <v>0.1625948</v>
       </c>
     </row>
     <row r="45">
@@ -2227,16 +2227,16 @@
         <v>3852.094</v>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0</v>
+        <v>10.35</v>
       </c>
       <c r="G45" s="5" t="n">
-        <v>0</v>
+        <v>0.556</v>
       </c>
       <c r="H45" s="6" t="n">
-        <v>0.1237076</v>
+        <v>0.1095627</v>
       </c>
       <c r="I45" s="6" t="n">
-        <v>0.1237076</v>
+        <v>0.1095627</v>
       </c>
     </row>
     <row r="46">
@@ -2258,16 +2258,16 @@
         <v>5719.531</v>
       </c>
       <c r="F46" s="5" t="n">
-        <v>0</v>
+        <v>13.58</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0</v>
+        <v>0.766</v>
       </c>
       <c r="H46" s="6" t="n">
-        <v>0.1260111</v>
+        <v>0.1237076</v>
       </c>
       <c r="I46" s="6" t="n">
-        <v>0.1260111</v>
+        <v>0.1237076</v>
       </c>
     </row>
     <row r="47">
@@ -2289,16 +2289,16 @@
         <v>5745</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>0</v>
+        <v>12.76</v>
       </c>
       <c r="G47" s="5" t="n">
-        <v>0</v>
+        <v>0.715</v>
       </c>
       <c r="H47" s="6" t="n">
-        <v>0.2611755</v>
+        <v>0.1260111</v>
       </c>
       <c r="I47" s="6" t="n">
-        <v>0.2611755</v>
+        <v>0.1260111</v>
       </c>
     </row>
     <row r="48">
@@ -2320,16 +2320,16 @@
         <v>5745</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>0</v>
+        <v>11.99</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0</v>
+        <v>0.669</v>
       </c>
       <c r="H48" s="6" t="n">
-        <v>0.2601367</v>
+        <v>0.2611755</v>
       </c>
       <c r="I48" s="6" t="n">
-        <v>0.2601367</v>
+        <v>0.2611755</v>
       </c>
     </row>
     <row r="49">
@@ -2351,16 +2351,16 @@
         <v>5746.5</v>
       </c>
       <c r="F49" s="5" t="n">
-        <v>0</v>
+        <v>11.43</v>
       </c>
       <c r="G49" s="5" t="n">
-        <v>0</v>
+        <v>0.623</v>
       </c>
       <c r="H49" s="6" t="n">
-        <v>0.1225956</v>
+        <v>0.2601367</v>
       </c>
       <c r="I49" s="6" t="n">
-        <v>0.1225956</v>
+        <v>0.2601367</v>
       </c>
     </row>
     <row r="50">
@@ -2382,16 +2382,16 @@
         <v>6988.969</v>
       </c>
       <c r="F50" s="5" t="n">
-        <v>0</v>
+        <v>16.78</v>
       </c>
       <c r="G50" s="5" t="n">
-        <v>0</v>
+        <v>0.715</v>
       </c>
       <c r="H50" s="6" t="n">
-        <v>0.2220208</v>
+        <v>0.1225956</v>
       </c>
       <c r="I50" s="6" t="n">
-        <v>0.2220208</v>
+        <v>0.1225956</v>
       </c>
     </row>
     <row r="51">
@@ -2413,16 +2413,16 @@
         <v>6991.578</v>
       </c>
       <c r="F51" s="5" t="n">
-        <v>0</v>
+        <v>15.97</v>
       </c>
       <c r="G51" s="5" t="n">
-        <v>0</v>
+        <v>0.679</v>
       </c>
       <c r="H51" s="6" t="n">
-        <v>0.2207892</v>
+        <v>0.2220208</v>
       </c>
       <c r="I51" s="6" t="n">
-        <v>0.2207892</v>
+        <v>0.2220208</v>
       </c>
     </row>
     <row r="52">
@@ -2444,16 +2444,16 @@
         <v>6991.641</v>
       </c>
       <c r="F52" s="5" t="n">
-        <v>0</v>
+        <v>15.19</v>
       </c>
       <c r="G52" s="5" t="n">
-        <v>0</v>
+        <v>0.644</v>
       </c>
       <c r="H52" s="6" t="n">
-        <v>0.1252291</v>
+        <v>0.2207892</v>
       </c>
       <c r="I52" s="6" t="n">
-        <v>0.1252291</v>
+        <v>0.2207892</v>
       </c>
     </row>
     <row r="53">
@@ -2475,16 +2475,16 @@
         <v>7006.094</v>
       </c>
       <c r="F53" s="5" t="n">
-        <v>0</v>
+        <v>14.87</v>
       </c>
       <c r="G53" s="5" t="n">
-        <v>0</v>
+        <v>0.613</v>
       </c>
       <c r="H53" s="6" t="n">
-        <v>0.184894</v>
+        <v>0.1252291</v>
       </c>
       <c r="I53" s="6" t="n">
-        <v>0.184894</v>
+        <v>0.1252291</v>
       </c>
     </row>
     <row r="54">
@@ -2506,16 +2506,16 @@
         <v>7016.375</v>
       </c>
       <c r="F54" s="5" t="n">
-        <v>0</v>
+        <v>14.33</v>
       </c>
       <c r="G54" s="5" t="n">
-        <v>0</v>
+        <v>0.588</v>
       </c>
       <c r="H54" s="6" t="n">
-        <v>0.2897047</v>
+        <v>0.184894</v>
       </c>
       <c r="I54" s="6" t="n">
-        <v>0.2897047</v>
+        <v>0.184894</v>
       </c>
     </row>
     <row r="55">
@@ -2537,16 +2537,16 @@
         <v>7033.703</v>
       </c>
       <c r="F55" s="5" t="n">
-        <v>0</v>
+        <v>13.64</v>
       </c>
       <c r="G55" s="5" t="n">
-        <v>0</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="H55" s="6" t="n">
-        <v>0.170116</v>
+        <v>0.2897047</v>
       </c>
       <c r="I55" s="6" t="n">
-        <v>0.170116</v>
+        <v>0.2897047</v>
       </c>
     </row>
     <row r="56">
@@ -2568,16 +2568,16 @@
         <v>7101.063</v>
       </c>
       <c r="F56" s="5" t="n">
-        <v>0</v>
+        <v>13.25</v>
       </c>
       <c r="G56" s="5" t="n">
-        <v>0</v>
+        <v>0.54</v>
       </c>
       <c r="H56" s="6" t="n">
-        <v>0.192526</v>
+        <v>0.170116</v>
       </c>
       <c r="I56" s="6" t="n">
-        <v>0.192526</v>
+        <v>0.170116</v>
       </c>
     </row>
     <row r="57">
@@ -2599,16 +2599,16 @@
         <v>7773.781</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>0</v>
+        <v>13.61</v>
       </c>
       <c r="G57" s="5" t="n">
-        <v>0</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="H57" s="6" t="n">
-        <v>0.2844053</v>
+        <v>0.192526</v>
       </c>
       <c r="I57" s="6" t="n">
-        <v>0.2844053</v>
+        <v>0.192526</v>
       </c>
     </row>
     <row r="58">
@@ -2630,16 +2630,16 @@
         <v>7776</v>
       </c>
       <c r="F58" s="5" t="n">
-        <v>0</v>
+        <v>13.05</v>
       </c>
       <c r="G58" s="5" t="n">
-        <v>0</v>
+        <v>0.541</v>
       </c>
       <c r="H58" s="6" t="n">
-        <v>0.2167756</v>
+        <v>0.2844053</v>
       </c>
       <c r="I58" s="6" t="n">
-        <v>0.2167756</v>
+        <v>0.2844053</v>
       </c>
     </row>
     <row r="59">
@@ -2661,16 +2661,16 @@
         <v>7776.063</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>0</v>
+        <v>12.55</v>
       </c>
       <c r="G59" s="5" t="n">
-        <v>0</v>
+        <v>0.52</v>
       </c>
       <c r="H59" s="6" t="n">
-        <v>0.2518649</v>
+        <v>0.2167756</v>
       </c>
       <c r="I59" s="6" t="n">
-        <v>0.2518649</v>
+        <v>0.2167756</v>
       </c>
     </row>
     <row r="60">
@@ -2692,16 +2692,16 @@
         <v>7776.063</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>0</v>
+        <v>12.12</v>
       </c>
       <c r="G60" s="5" t="n">
-        <v>0</v>
+        <v>0.501</v>
       </c>
       <c r="H60" s="6" t="n">
-        <v>0.2300291</v>
+        <v>0.2518649</v>
       </c>
       <c r="I60" s="6" t="n">
-        <v>0.2300291</v>
+        <v>0.2518649</v>
       </c>
     </row>
     <row r="61">
@@ -2723,16 +2723,16 @@
         <v>7783.969</v>
       </c>
       <c r="F61" s="5" t="n">
-        <v>0</v>
+        <v>11.76</v>
       </c>
       <c r="G61" s="5" t="n">
-        <v>0</v>
+        <v>0.484</v>
       </c>
       <c r="H61" s="6" t="n">
-        <v>0.2498192</v>
+        <v>0.2300291</v>
       </c>
       <c r="I61" s="6" t="n">
-        <v>0.2498192</v>
+        <v>0.2300291</v>
       </c>
     </row>
     <row r="62">
@@ -2754,16 +2754,16 @@
         <v>7784.547</v>
       </c>
       <c r="F62" s="5" t="n">
-        <v>0</v>
+        <v>11.36</v>
       </c>
       <c r="G62" s="5" t="n">
-        <v>0</v>
+        <v>0.467</v>
       </c>
       <c r="H62" s="6" t="n">
-        <v>0.1102495</v>
+        <v>0.2498192</v>
       </c>
       <c r="I62" s="6" t="n">
-        <v>0.1102495</v>
+        <v>0.2498192</v>
       </c>
     </row>
     <row r="63">
@@ -2785,16 +2785,16 @@
         <v>7842.109</v>
       </c>
       <c r="F63" s="5" t="n">
-        <v>0</v>
+        <v>11.05</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>0</v>
+        <v>0.454</v>
       </c>
       <c r="H63" s="6" t="n">
-        <v>0</v>
+        <v>0.1102495</v>
       </c>
       <c r="I63" s="6" t="n">
-        <v>0</v>
+        <v>0.1102495</v>
       </c>
     </row>
     <row r="64">
@@ -2816,10 +2816,10 @@
         <v>21.188</v>
       </c>
       <c r="F64" s="5" t="n">
-        <v>0</v>
+        <v>1.99</v>
       </c>
       <c r="G64" s="5" t="n">
-        <v>0</v>
+        <v>0.038</v>
       </c>
       <c r="H64" s="6" t="n">
         <v>0.1260111</v>
@@ -2847,16 +2847,16 @@
         <v>61.344</v>
       </c>
       <c r="F65" s="5" t="n">
-        <v>0</v>
+        <v>1.61</v>
       </c>
       <c r="G65" s="5" t="n">
-        <v>0</v>
+        <v>0.052</v>
       </c>
       <c r="H65" s="6" t="n">
-        <v>0.2289273</v>
+        <v>0.1260111</v>
       </c>
       <c r="I65" s="6" t="n">
-        <v>0.2289273</v>
+        <v>0.1260111</v>
       </c>
     </row>
     <row r="66">
@@ -2878,16 +2878,16 @@
         <v>61.516</v>
       </c>
       <c r="F66" s="5" t="n">
-        <v>0</v>
+        <v>1.42</v>
       </c>
       <c r="G66" s="5" t="n">
-        <v>0</v>
+        <v>0.035</v>
       </c>
       <c r="H66" s="6" t="n">
-        <v>0.199396</v>
+        <v>0.2289273</v>
       </c>
       <c r="I66" s="6" t="n">
-        <v>0.199396</v>
+        <v>0.2289273</v>
       </c>
     </row>
     <row r="67">
@@ -2909,16 +2909,16 @@
         <v>61.703</v>
       </c>
       <c r="F67" s="5" t="n">
-        <v>0</v>
+        <v>1.14</v>
       </c>
       <c r="G67" s="5" t="n">
-        <v>0</v>
+        <v>0.027</v>
       </c>
       <c r="H67" s="6" t="n">
-        <v>0.192526</v>
+        <v>0.199396</v>
       </c>
       <c r="I67" s="6" t="n">
-        <v>0.192526</v>
+        <v>0.199396</v>
       </c>
     </row>
     <row r="68">
@@ -2940,16 +2940,16 @@
         <v>177.078</v>
       </c>
       <c r="F68" s="5" t="n">
-        <v>0</v>
+        <v>2.84</v>
       </c>
       <c r="G68" s="5" t="n">
-        <v>0</v>
+        <v>0.063</v>
       </c>
       <c r="H68" s="6" t="n">
-        <v>0.1624159</v>
+        <v>0.192526</v>
       </c>
       <c r="I68" s="6" t="n">
-        <v>0.1624159</v>
+        <v>0.192526</v>
       </c>
     </row>
     <row r="69">
@@ -2971,16 +2971,16 @@
         <v>327.453</v>
       </c>
       <c r="F69" s="5" t="n">
-        <v>0</v>
+        <v>10.51</v>
       </c>
       <c r="G69" s="5" t="n">
-        <v>0</v>
+        <v>0.098</v>
       </c>
       <c r="H69" s="6" t="n">
-        <v>0.1985302</v>
+        <v>0.1624159</v>
       </c>
       <c r="I69" s="6" t="n">
-        <v>0.1985302</v>
+        <v>0.1624159</v>
       </c>
     </row>
     <row r="70">
@@ -3002,16 +3002,16 @@
         <v>381.141</v>
       </c>
       <c r="F70" s="5" t="n">
-        <v>0</v>
+        <v>9.48</v>
       </c>
       <c r="G70" s="5" t="n">
-        <v>0</v>
+        <v>0.098</v>
       </c>
       <c r="H70" s="6" t="n">
-        <v>0.2313895</v>
+        <v>0.1985302</v>
       </c>
       <c r="I70" s="6" t="n">
-        <v>0.2313895</v>
+        <v>0.1985302</v>
       </c>
     </row>
     <row r="71">
@@ -3033,16 +3033,16 @@
         <v>393.484</v>
       </c>
       <c r="F71" s="5" t="n">
-        <v>0</v>
+        <v>8.41</v>
       </c>
       <c r="G71" s="5" t="n">
-        <v>0</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="H71" s="6" t="n">
-        <v>0.233184</v>
+        <v>0.2313895</v>
       </c>
       <c r="I71" s="6" t="n">
-        <v>0.233184</v>
+        <v>0.2313895</v>
       </c>
     </row>
     <row r="72">
@@ -3064,16 +3064,16 @@
         <v>393.484</v>
       </c>
       <c r="F72" s="5" t="n">
-        <v>0</v>
+        <v>7.46</v>
       </c>
       <c r="G72" s="5" t="n">
-        <v>0</v>
+        <v>0.078</v>
       </c>
       <c r="H72" s="6" t="n">
-        <v>0.1201376</v>
+        <v>0.233184</v>
       </c>
       <c r="I72" s="6" t="n">
-        <v>0.1201376</v>
+        <v>0.233184</v>
       </c>
     </row>
     <row r="73">
@@ -3095,16 +3095,16 @@
         <v>4808.094</v>
       </c>
       <c r="F73" s="5" t="n">
-        <v>0</v>
+        <v>16.91</v>
       </c>
       <c r="G73" s="5" t="n">
-        <v>0</v>
+        <v>0.862</v>
       </c>
       <c r="H73" s="6" t="n">
-        <v>0.1229662</v>
+        <v>0.1201376</v>
       </c>
       <c r="I73" s="6" t="n">
-        <v>0.1229662</v>
+        <v>0.1201376</v>
       </c>
     </row>
     <row r="74">
@@ -3126,16 +3126,16 @@
         <v>4865.203</v>
       </c>
       <c r="F74" s="5" t="n">
-        <v>0</v>
+        <v>15.37</v>
       </c>
       <c r="G74" s="5" t="n">
-        <v>0</v>
+        <v>0.785</v>
       </c>
       <c r="H74" s="6" t="n">
-        <v>0.2826314</v>
+        <v>0.1229662</v>
       </c>
       <c r="I74" s="6" t="n">
-        <v>0.2826314</v>
+        <v>0.1229662</v>
       </c>
     </row>
     <row r="75">
@@ -3157,16 +3157,16 @@
         <v>4865.516</v>
       </c>
       <c r="F75" s="5" t="n">
-        <v>0</v>
+        <v>14.12</v>
       </c>
       <c r="G75" s="5" t="n">
-        <v>0</v>
+        <v>0.718</v>
       </c>
       <c r="H75" s="6" t="n">
-        <v>0.2844053</v>
+        <v>0.2826314</v>
       </c>
       <c r="I75" s="6" t="n">
-        <v>0.2844053</v>
+        <v>0.2826314</v>
       </c>
     </row>
     <row r="76">
@@ -3188,10 +3188,10 @@
         <v>4877.359</v>
       </c>
       <c r="F76" s="5" t="n">
-        <v>0</v>
+        <v>13.15</v>
       </c>
       <c r="G76" s="5" t="n">
-        <v>0</v>
+        <v>0.663</v>
       </c>
       <c r="H76" s="6" t="n">
         <v>0.2844053</v>
@@ -3219,16 +3219,16 @@
         <v>4880.266</v>
       </c>
       <c r="F77" s="5" t="n">
-        <v>0</v>
+        <v>12.24</v>
       </c>
       <c r="G77" s="5" t="n">
-        <v>0</v>
+        <v>0.616</v>
       </c>
       <c r="H77" s="6" t="n">
-        <v>0.1880851</v>
+        <v>0.2844053</v>
       </c>
       <c r="I77" s="6" t="n">
-        <v>0.1880851</v>
+        <v>0.2844053</v>
       </c>
     </row>
     <row r="78">
@@ -3250,16 +3250,16 @@
         <v>4880.906</v>
       </c>
       <c r="F78" s="5" t="n">
-        <v>0</v>
+        <v>11.37</v>
       </c>
       <c r="G78" s="5" t="n">
-        <v>0</v>
+        <v>0.571</v>
       </c>
       <c r="H78" s="6" t="n">
-        <v>0.1033878</v>
+        <v>0.1880851</v>
       </c>
       <c r="I78" s="6" t="n">
-        <v>0.1033878</v>
+        <v>0.1880851</v>
       </c>
     </row>
     <row r="79">
@@ -3281,16 +3281,16 @@
         <v>4907.063</v>
       </c>
       <c r="F79" s="5" t="n">
-        <v>0</v>
+        <v>10.65</v>
       </c>
       <c r="G79" s="5" t="n">
-        <v>0</v>
+        <v>0.53</v>
       </c>
       <c r="H79" s="6" t="n">
-        <v>0.1060832</v>
+        <v>0.1033878</v>
       </c>
       <c r="I79" s="6" t="n">
-        <v>0.1060832</v>
+        <v>0.1033878</v>
       </c>
     </row>
     <row r="80">
@@ -3312,16 +3312,16 @@
         <v>11341.281</v>
       </c>
       <c r="F80" s="5" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="G80" s="5" t="n">
-        <v>0</v>
+        <v>1.15</v>
       </c>
       <c r="H80" s="6" t="n">
-        <v>0.0917698</v>
+        <v>0.1060832</v>
       </c>
       <c r="I80" s="6" t="n">
-        <v>0.0917698</v>
+        <v>0.1060832</v>
       </c>
     </row>
     <row r="81">
@@ -3343,16 +3343,16 @@
         <v>12569.578</v>
       </c>
       <c r="F81" s="5" t="n">
-        <v>0</v>
+        <v>17.01</v>
       </c>
       <c r="G81" s="5" t="n">
-        <v>0</v>
+        <v>1.202</v>
       </c>
       <c r="H81" s="6" t="n">
-        <v>0.2272512</v>
+        <v>0.0917698</v>
       </c>
       <c r="I81" s="6" t="n">
-        <v>0.2272512</v>
+        <v>0.0917698</v>
       </c>
     </row>
     <row r="82">
@@ -3374,16 +3374,16 @@
         <v>12603.969</v>
       </c>
       <c r="F82" s="5" t="n">
-        <v>0</v>
+        <v>16.25</v>
       </c>
       <c r="G82" s="5" t="n">
-        <v>0</v>
+        <v>1.146</v>
       </c>
       <c r="H82" s="6" t="n">
-        <v>0.1987498</v>
+        <v>0.2272512</v>
       </c>
       <c r="I82" s="6" t="n">
-        <v>0.1987498</v>
+        <v>0.2272512</v>
       </c>
     </row>
     <row r="83">
@@ -3405,16 +3405,16 @@
         <v>12606.875</v>
       </c>
       <c r="F83" s="5" t="n">
-        <v>0</v>
+        <v>15.45</v>
       </c>
       <c r="G83" s="5" t="n">
-        <v>0</v>
+        <v>1.087</v>
       </c>
       <c r="H83" s="6" t="n">
-        <v>0.201175</v>
+        <v>0.1987498</v>
       </c>
       <c r="I83" s="6" t="n">
-        <v>0.201175</v>
+        <v>0.1987498</v>
       </c>
     </row>
     <row r="84">
@@ -3436,16 +3436,16 @@
         <v>12620.625</v>
       </c>
       <c r="F84" s="5" t="n">
-        <v>0</v>
+        <v>14.8</v>
       </c>
       <c r="G84" s="5" t="n">
-        <v>0</v>
+        <v>1.039</v>
       </c>
       <c r="H84" s="6" t="n">
-        <v>0.2186665</v>
+        <v>0.201175</v>
       </c>
       <c r="I84" s="6" t="n">
-        <v>0.2186665</v>
+        <v>0.201175</v>
       </c>
     </row>
     <row r="85">
@@ -3467,16 +3467,16 @@
         <v>12623.547</v>
       </c>
       <c r="F85" s="5" t="n">
-        <v>0</v>
+        <v>14.21</v>
       </c>
       <c r="G85" s="5" t="n">
-        <v>0</v>
+        <v>0.997</v>
       </c>
       <c r="H85" s="6" t="n">
-        <v>0.2634557</v>
+        <v>0.2186665</v>
       </c>
       <c r="I85" s="6" t="n">
-        <v>0.2634557</v>
+        <v>0.2186665</v>
       </c>
     </row>
     <row r="86">
@@ -3498,16 +3498,16 @@
         <v>12636.344</v>
       </c>
       <c r="F86" s="5" t="n">
-        <v>0</v>
+        <v>13.6</v>
       </c>
       <c r="G86" s="5" t="n">
-        <v>0</v>
+        <v>0.951</v>
       </c>
       <c r="H86" s="6" t="n">
-        <v>0.2184949</v>
+        <v>0.2634557</v>
       </c>
       <c r="I86" s="6" t="n">
-        <v>0.2184949</v>
+        <v>0.2634557</v>
       </c>
     </row>
     <row r="87">
@@ -3529,16 +3529,16 @@
         <v>13554.313</v>
       </c>
       <c r="F87" s="5" t="n">
-        <v>0</v>
+        <v>13.93</v>
       </c>
       <c r="G87" s="5" t="n">
-        <v>0</v>
+        <v>0.975</v>
       </c>
       <c r="H87" s="6" t="n">
-        <v>0.2258766</v>
+        <v>0.2184949</v>
       </c>
       <c r="I87" s="6" t="n">
-        <v>0.2258766</v>
+        <v>0.2184949</v>
       </c>
     </row>
     <row r="88">
@@ -3560,16 +3560,16 @@
         <v>13555.188</v>
       </c>
       <c r="F88" s="5" t="n">
-        <v>0</v>
+        <v>13.43</v>
       </c>
       <c r="G88" s="5" t="n">
-        <v>0</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="H88" s="6" t="n">
-        <v>0.2176948</v>
+        <v>0.2258766</v>
       </c>
       <c r="I88" s="6" t="n">
-        <v>0.2176948</v>
+        <v>0.2258766</v>
       </c>
     </row>
     <row r="89">
@@ -3591,16 +3591,16 @@
         <v>13558.016</v>
       </c>
       <c r="F89" s="5" t="n">
-        <v>0</v>
+        <v>12.87</v>
       </c>
       <c r="G89" s="5" t="n">
-        <v>0</v>
+        <v>0.898</v>
       </c>
       <c r="H89" s="6" t="n">
-        <v>0.208873</v>
+        <v>0.2176948</v>
       </c>
       <c r="I89" s="6" t="n">
-        <v>0.208873</v>
+        <v>0.2176948</v>
       </c>
     </row>
     <row r="90">
@@ -3622,16 +3622,16 @@
         <v>13564.25</v>
       </c>
       <c r="F90" s="5" t="n">
-        <v>0</v>
+        <v>12.42</v>
       </c>
       <c r="G90" s="5" t="n">
-        <v>0</v>
+        <v>0.866</v>
       </c>
       <c r="H90" s="6" t="n">
-        <v>0.2844053</v>
+        <v>0.208873</v>
       </c>
       <c r="I90" s="6" t="n">
-        <v>0.2844053</v>
+        <v>0.208873</v>
       </c>
     </row>
     <row r="91">
@@ -3653,10 +3653,10 @@
         <v>13564.25</v>
       </c>
       <c r="F91" s="5" t="n">
-        <v>0</v>
+        <v>12.02</v>
       </c>
       <c r="G91" s="5" t="n">
-        <v>0</v>
+        <v>0.835</v>
       </c>
       <c r="H91" s="6" t="n">
         <v>0.2844053</v>
@@ -3684,16 +3684,16 @@
         <v>13569.688</v>
       </c>
       <c r="F92" s="5" t="n">
-        <v>0</v>
+        <v>11.54</v>
       </c>
       <c r="G92" s="5" t="n">
-        <v>0</v>
+        <v>0.798</v>
       </c>
       <c r="H92" s="6" t="n">
-        <v>0.1918669</v>
+        <v>0.2844053</v>
       </c>
       <c r="I92" s="6" t="n">
-        <v>0.1918669</v>
+        <v>0.2844053</v>
       </c>
     </row>
     <row r="93">
@@ -3715,16 +3715,16 @@
         <v>13710.688</v>
       </c>
       <c r="F93" s="5" t="n">
-        <v>0</v>
+        <v>11.27</v>
       </c>
       <c r="G93" s="5" t="n">
-        <v>0</v>
+        <v>0.779</v>
       </c>
       <c r="H93" s="6" t="n">
-        <v>0</v>
+        <v>0.1918669</v>
       </c>
       <c r="I93" s="6" t="n">
-        <v>0</v>
+        <v>0.1918669</v>
       </c>
     </row>
     <row r="94">
@@ -3746,16 +3746,16 @@
         <v>1.313</v>
       </c>
       <c r="F94" s="5" t="n">
-        <v>0</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="G94" s="5" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="H94" s="6" t="n">
-        <v>0.2509308</v>
+        <v>0.2198847</v>
       </c>
       <c r="I94" s="6" t="n">
-        <v>0.2509308</v>
+        <v>0.2198847</v>
       </c>
     </row>
     <row r="95">
@@ -3777,16 +3777,16 @@
         <v>10.969</v>
       </c>
       <c r="F95" s="5" t="n">
-        <v>0</v>
+        <v>1.13</v>
       </c>
       <c r="G95" s="5" t="n">
-        <v>0</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="H95" s="6" t="n">
-        <v>0.2098487</v>
+        <v>0.2509308</v>
       </c>
       <c r="I95" s="6" t="n">
-        <v>0.2098487</v>
+        <v>0.2509308</v>
       </c>
     </row>
     <row r="96">
@@ -3808,16 +3808,16 @@
         <v>38.016</v>
       </c>
       <c r="F96" s="5" t="n">
-        <v>0</v>
+        <v>1.04</v>
       </c>
       <c r="G96" s="5" t="n">
-        <v>0</v>
+        <v>0.021</v>
       </c>
       <c r="H96" s="6" t="n">
-        <v>0.2110814</v>
+        <v>0.2098487</v>
       </c>
       <c r="I96" s="6" t="n">
-        <v>0.2110814</v>
+        <v>0.2098487</v>
       </c>
     </row>
     <row r="97">
@@ -3839,16 +3839,16 @@
         <v>48.266</v>
       </c>
       <c r="F97" s="5" t="n">
-        <v>0</v>
+        <v>0.93</v>
       </c>
       <c r="G97" s="5" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="H97" s="6" t="n">
-        <v>0.2641469</v>
+        <v>0.2110814</v>
       </c>
       <c r="I97" s="6" t="n">
-        <v>0.2641469</v>
+        <v>0.2110814</v>
       </c>
     </row>
     <row r="98">
@@ -3870,16 +3870,16 @@
         <v>328.75</v>
       </c>
       <c r="F98" s="5" t="n">
-        <v>0</v>
+        <v>1.47</v>
       </c>
       <c r="G98" s="5" t="n">
-        <v>0</v>
+        <v>0.11</v>
       </c>
       <c r="H98" s="6" t="n">
-        <v>0.2788382</v>
+        <v>0.2641469</v>
       </c>
       <c r="I98" s="6" t="n">
-        <v>0.2788382</v>
+        <v>0.2641469</v>
       </c>
     </row>
     <row r="99">
@@ -3901,16 +3901,16 @@
         <v>347.719</v>
       </c>
       <c r="F99" s="5" t="n">
-        <v>0</v>
+        <v>1.37</v>
       </c>
       <c r="G99" s="5" t="n">
-        <v>0</v>
+        <v>0.098</v>
       </c>
       <c r="H99" s="6" t="n">
-        <v>0.1232496</v>
+        <v>0.2788382</v>
       </c>
       <c r="I99" s="6" t="n">
-        <v>0.1232496</v>
+        <v>0.2788382</v>
       </c>
     </row>
     <row r="100">
@@ -3932,16 +3932,16 @@
         <v>3465.188</v>
       </c>
       <c r="F100" s="5" t="n">
-        <v>0</v>
+        <v>7.01</v>
       </c>
       <c r="G100" s="5" t="n">
-        <v>0</v>
+        <v>0.848</v>
       </c>
       <c r="H100" s="6" t="n">
-        <v>0.2617761</v>
+        <v>0.1232496</v>
       </c>
       <c r="I100" s="6" t="n">
-        <v>0.2617761</v>
+        <v>0.1232496</v>
       </c>
     </row>
     <row r="101">
@@ -3963,16 +3963,16 @@
         <v>3465.406</v>
       </c>
       <c r="F101" s="5" t="n">
-        <v>0</v>
+        <v>6.11</v>
       </c>
       <c r="G101" s="5" t="n">
-        <v>0</v>
+        <v>0.733</v>
       </c>
       <c r="H101" s="6" t="n">
-        <v>0.1838224</v>
+        <v>0.2617761</v>
       </c>
       <c r="I101" s="6" t="n">
-        <v>0.1838224</v>
+        <v>0.2617761</v>
       </c>
     </row>
     <row r="102">
@@ -3994,16 +3994,16 @@
         <v>3479.125</v>
       </c>
       <c r="F102" s="5" t="n">
-        <v>0</v>
+        <v>5.54</v>
       </c>
       <c r="G102" s="5" t="n">
-        <v>0</v>
+        <v>0.654</v>
       </c>
       <c r="H102" s="6" t="n">
-        <v>0.1218389</v>
+        <v>0.1838224</v>
       </c>
       <c r="I102" s="6" t="n">
-        <v>0.1218389</v>
+        <v>0.1838224</v>
       </c>
     </row>
     <row r="103">
@@ -4025,16 +4025,16 @@
         <v>9230.422</v>
       </c>
       <c r="F103" s="5" t="n">
-        <v>0</v>
+        <v>13.09</v>
       </c>
       <c r="G103" s="5" t="n">
-        <v>0</v>
+        <v>1.571</v>
       </c>
       <c r="H103" s="6" t="n">
-        <v>0.2667958</v>
+        <v>0.1218389</v>
       </c>
       <c r="I103" s="6" t="n">
-        <v>0.2667958</v>
+        <v>0.1218389</v>
       </c>
     </row>
     <row r="104">
@@ -4056,16 +4056,16 @@
         <v>9230.422</v>
       </c>
       <c r="F104" s="5" t="n">
-        <v>0</v>
+        <v>11.99</v>
       </c>
       <c r="G104" s="5" t="n">
-        <v>0</v>
+        <v>1.437</v>
       </c>
       <c r="H104" s="6" t="n">
-        <v>0.2183271</v>
+        <v>0.2667958</v>
       </c>
       <c r="I104" s="6" t="n">
-        <v>0.2183271</v>
+        <v>0.2667958</v>
       </c>
     </row>
     <row r="105">
@@ -4087,16 +4087,16 @@
         <v>9235.172</v>
       </c>
       <c r="F105" s="5" t="n">
-        <v>0</v>
+        <v>11.06</v>
       </c>
       <c r="G105" s="5" t="n">
-        <v>0</v>
+        <v>1.319</v>
       </c>
       <c r="H105" s="6" t="n">
-        <v>0.1704796</v>
+        <v>0.2183271</v>
       </c>
       <c r="I105" s="6" t="n">
-        <v>0.1704796</v>
+        <v>0.2183271</v>
       </c>
     </row>
     <row r="106">
@@ -4118,16 +4118,16 @@
         <v>9250.531000000001</v>
       </c>
       <c r="F106" s="5" t="n">
-        <v>0</v>
+        <v>10.27</v>
       </c>
       <c r="G106" s="5" t="n">
-        <v>0</v>
+        <v>1.216</v>
       </c>
       <c r="H106" s="6" t="n">
-        <v>0.2498192</v>
+        <v>0.1704796</v>
       </c>
       <c r="I106" s="6" t="n">
-        <v>0.2498192</v>
+        <v>0.1704796</v>
       </c>
     </row>
     <row r="107">
@@ -4149,16 +4149,16 @@
         <v>9258.188</v>
       </c>
       <c r="F107" s="5" t="n">
-        <v>0</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="G107" s="5" t="n">
-        <v>0</v>
+        <v>1.129</v>
       </c>
       <c r="H107" s="6" t="n">
-        <v>0.1838224</v>
+        <v>0.2498192</v>
       </c>
       <c r="I107" s="6" t="n">
-        <v>0.1838224</v>
+        <v>0.2498192</v>
       </c>
     </row>
     <row r="108">
@@ -4180,16 +4180,16 @@
         <v>9394.25</v>
       </c>
       <c r="F108" s="5" t="n">
-        <v>0</v>
+        <v>9.07</v>
       </c>
       <c r="G108" s="5" t="n">
-        <v>0</v>
+        <v>1.067</v>
       </c>
       <c r="H108" s="6" t="n">
-        <v>0.1920985</v>
+        <v>0.1838224</v>
       </c>
       <c r="I108" s="6" t="n">
-        <v>0.1920985</v>
+        <v>0.1838224</v>
       </c>
     </row>
     <row r="109">
@@ -4211,16 +4211,16 @@
         <v>9394.468999999999</v>
       </c>
       <c r="F109" s="5" t="n">
-        <v>0</v>
+        <v>8.58</v>
       </c>
       <c r="G109" s="5" t="n">
-        <v>0</v>
+        <v>1.005</v>
       </c>
       <c r="H109" s="6" t="n">
-        <v>0.1146563</v>
+        <v>0.1920985</v>
       </c>
       <c r="I109" s="6" t="n">
-        <v>0.1146563</v>
+        <v>0.1920985</v>
       </c>
     </row>
     <row r="110">
@@ -4242,16 +4242,16 @@
         <v>13801.844</v>
       </c>
       <c r="F110" s="5" t="n">
-        <v>0</v>
+        <v>12.04</v>
       </c>
       <c r="G110" s="5" t="n">
-        <v>0</v>
+        <v>1.385</v>
       </c>
       <c r="H110" s="6" t="n">
-        <v>0.1980923</v>
+        <v>0.1146563</v>
       </c>
       <c r="I110" s="6" t="n">
-        <v>0.1980923</v>
+        <v>0.1146563</v>
       </c>
     </row>
     <row r="111">
@@ -4273,16 +4273,16 @@
         <v>13813.891</v>
       </c>
       <c r="F111" s="5" t="n">
-        <v>0</v>
+        <v>11.46</v>
       </c>
       <c r="G111" s="5" t="n">
-        <v>0</v>
+        <v>1.313</v>
       </c>
       <c r="H111" s="6" t="n">
-        <v>0.2844053</v>
+        <v>0.1980923</v>
       </c>
       <c r="I111" s="6" t="n">
-        <v>0.2844053</v>
+        <v>0.1980923</v>
       </c>
     </row>
     <row r="112">
@@ -4304,16 +4304,16 @@
         <v>13814.109</v>
       </c>
       <c r="F112" s="5" t="n">
-        <v>0</v>
+        <v>10.9</v>
       </c>
       <c r="G112" s="5" t="n">
-        <v>0</v>
+        <v>1.245</v>
       </c>
       <c r="H112" s="6" t="n">
-        <v>0.1395497</v>
+        <v>0.2844053</v>
       </c>
       <c r="I112" s="6" t="n">
-        <v>0.1395497</v>
+        <v>0.2844053</v>
       </c>
     </row>
     <row r="113">
@@ -4335,16 +4335,16 @@
         <v>13829.688</v>
       </c>
       <c r="F113" s="5" t="n">
-        <v>0</v>
+        <v>10.29</v>
       </c>
       <c r="G113" s="5" t="n">
-        <v>0</v>
+        <v>1.172</v>
       </c>
       <c r="H113" s="6" t="n">
-        <v>0.2235431</v>
+        <v>0.1395497</v>
       </c>
       <c r="I113" s="6" t="n">
-        <v>0.2235431</v>
+        <v>0.1395497</v>
       </c>
     </row>
     <row r="114">
@@ -4366,16 +4366,16 @@
         <v>13831.234</v>
       </c>
       <c r="F114" s="5" t="n">
-        <v>0</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="G114" s="5" t="n">
-        <v>0</v>
+        <v>1.113</v>
       </c>
       <c r="H114" s="6" t="n">
-        <v>0.2844053</v>
+        <v>0.2235431</v>
       </c>
       <c r="I114" s="6" t="n">
-        <v>0.2844053</v>
+        <v>0.2235431</v>
       </c>
     </row>
     <row r="115">
@@ -4397,16 +4397,16 @@
         <v>13832.281</v>
       </c>
       <c r="F115" s="5" t="n">
-        <v>0</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="G115" s="5" t="n">
-        <v>0</v>
+        <v>1.064</v>
       </c>
       <c r="H115" s="6" t="n">
-        <v>0.2285513</v>
+        <v>0.2844053</v>
       </c>
       <c r="I115" s="6" t="n">
-        <v>0.2285513</v>
+        <v>0.2844053</v>
       </c>
     </row>
     <row r="116">
@@ -4428,16 +4428,16 @@
         <v>13837.453</v>
       </c>
       <c r="F116" s="5" t="n">
-        <v>0</v>
+        <v>9.02</v>
       </c>
       <c r="G116" s="5" t="n">
-        <v>0</v>
+        <v>1.022</v>
       </c>
       <c r="H116" s="6" t="n">
-        <v>0.2633335</v>
+        <v>0.2285513</v>
       </c>
       <c r="I116" s="6" t="n">
-        <v>0.2633335</v>
+        <v>0.2285513</v>
       </c>
     </row>
     <row r="117">
@@ -4459,16 +4459,16 @@
         <v>13841.266</v>
       </c>
       <c r="F117" s="5" t="n">
-        <v>0</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G117" s="5" t="n">
-        <v>0</v>
+        <v>0.981</v>
       </c>
       <c r="H117" s="6" t="n">
-        <v>0.2755141</v>
+        <v>0.2633335</v>
       </c>
       <c r="I117" s="6" t="n">
-        <v>0.2755141</v>
+        <v>0.2633335</v>
       </c>
     </row>
     <row r="118">
@@ -4490,16 +4490,16 @@
         <v>13857.031</v>
       </c>
       <c r="F118" s="5" t="n">
-        <v>0</v>
+        <v>8.4</v>
       </c>
       <c r="G118" s="5" t="n">
-        <v>0</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="H118" s="6" t="n">
-        <v>0.2663427</v>
+        <v>0.2755141</v>
       </c>
       <c r="I118" s="6" t="n">
-        <v>0.2663427</v>
+        <v>0.2755141</v>
       </c>
     </row>
     <row r="119">
@@ -4521,16 +4521,16 @@
         <v>13862.172</v>
       </c>
       <c r="F119" s="5" t="n">
-        <v>0</v>
+        <v>8.09</v>
       </c>
       <c r="G119" s="5" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="H119" s="6" t="n">
-        <v>0.1870038</v>
+        <v>0.2663427</v>
       </c>
       <c r="I119" s="6" t="n">
-        <v>0.1870038</v>
+        <v>0.2663427</v>
       </c>
     </row>
     <row r="120">
@@ -4552,16 +4552,16 @@
         <v>15375.422</v>
       </c>
       <c r="F120" s="5" t="n">
-        <v>0</v>
+        <v>8.43</v>
       </c>
       <c r="G120" s="5" t="n">
-        <v>0</v>
+        <v>0.961</v>
       </c>
       <c r="H120" s="6" t="n">
-        <v>0.2487015</v>
+        <v>0.1870038</v>
       </c>
       <c r="I120" s="6" t="n">
-        <v>0.2487015</v>
+        <v>0.1870038</v>
       </c>
     </row>
     <row r="121">
@@ -4583,16 +4583,16 @@
         <v>15375.5</v>
       </c>
       <c r="F121" s="5" t="n">
-        <v>0</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="G121" s="5" t="n">
-        <v>0</v>
+        <v>0.927</v>
       </c>
       <c r="H121" s="6" t="n">
-        <v>0.119323</v>
+        <v>0.2487015</v>
       </c>
       <c r="I121" s="6" t="n">
-        <v>0.119323</v>
+        <v>0.2487015</v>
       </c>
     </row>
     <row r="122">
@@ -4614,16 +4614,16 @@
         <v>18359.891</v>
       </c>
       <c r="F122" s="5" t="n">
-        <v>0</v>
+        <v>9.23</v>
       </c>
       <c r="G122" s="5" t="n">
-        <v>0</v>
+        <v>1.068</v>
       </c>
       <c r="H122" s="6" t="n">
-        <v>0.2213283</v>
+        <v>0.119323</v>
       </c>
       <c r="I122" s="6" t="n">
-        <v>0.2213283</v>
+        <v>0.119323</v>
       </c>
     </row>
     <row r="123">
@@ -4645,16 +4645,16 @@
         <v>18364.703</v>
       </c>
       <c r="F123" s="5" t="n">
-        <v>0</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="G123" s="5" t="n">
-        <v>0</v>
+        <v>1.034</v>
       </c>
       <c r="H123" s="6" t="n">
-        <v>0</v>
+        <v>0.2213283</v>
       </c>
       <c r="I123" s="6" t="n">
-        <v>0</v>
+        <v>0.2213283</v>
       </c>
     </row>
     <row r="124">
@@ -4676,16 +4676,16 @@
         <v>0.188</v>
       </c>
       <c r="F124" s="5" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="G124" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H124" s="6" t="n">
-        <v>0.2707355</v>
+        <v>0.2844053</v>
       </c>
       <c r="I124" s="6" t="n">
-        <v>0.2707355</v>
+        <v>0.2844053</v>
       </c>
     </row>
     <row r="125">
@@ -4707,16 +4707,16 @@
         <v>7.328</v>
       </c>
       <c r="F125" s="5" t="n">
-        <v>0</v>
+        <v>0.37</v>
       </c>
       <c r="G125" s="5" t="n">
-        <v>0</v>
+        <v>0.006</v>
       </c>
       <c r="H125" s="6" t="n">
-        <v>0.2844053</v>
+        <v>0.2707355</v>
       </c>
       <c r="I125" s="6" t="n">
-        <v>0.2844053</v>
+        <v>0.2707355</v>
       </c>
     </row>
     <row r="126">
@@ -4738,16 +4738,16 @@
         <v>7.703</v>
       </c>
       <c r="F126" s="5" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="G126" s="5" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="H126" s="6" t="n">
-        <v>0.2263391</v>
+        <v>0.2844053</v>
       </c>
       <c r="I126" s="6" t="n">
-        <v>0.2263391</v>
+        <v>0.2844053</v>
       </c>
     </row>
     <row r="127">
@@ -4769,16 +4769,16 @@
         <v>7.703</v>
       </c>
       <c r="F127" s="5" t="n">
-        <v>0</v>
+        <v>0.51</v>
       </c>
       <c r="G127" s="5" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="H127" s="6" t="n">
-        <v>0.1161702</v>
+        <v>0.2263391</v>
       </c>
       <c r="I127" s="6" t="n">
-        <v>0.1161702</v>
+        <v>0.2263391</v>
       </c>
     </row>
     <row r="128">
@@ -4800,16 +4800,16 @@
         <v>1582.563</v>
       </c>
       <c r="F128" s="5" t="n">
-        <v>0</v>
+        <v>3.24</v>
       </c>
       <c r="G128" s="5" t="n">
-        <v>0</v>
+        <v>0.525</v>
       </c>
       <c r="H128" s="6" t="n">
-        <v>0.2195415</v>
+        <v>0.1161702</v>
       </c>
       <c r="I128" s="6" t="n">
-        <v>0.2195415</v>
+        <v>0.1161702</v>
       </c>
     </row>
     <row r="129">
@@ -4831,16 +4831,16 @@
         <v>1582.766</v>
       </c>
       <c r="F129" s="5" t="n">
-        <v>0</v>
+        <v>2.77</v>
       </c>
       <c r="G129" s="5" t="n">
-        <v>0</v>
+        <v>0.433</v>
       </c>
       <c r="H129" s="6" t="n">
-        <v>0.2489028</v>
+        <v>0.2195415</v>
       </c>
       <c r="I129" s="6" t="n">
-        <v>0.2489028</v>
+        <v>0.2195415</v>
       </c>
     </row>
     <row r="130">
@@ -4862,16 +4862,16 @@
         <v>1655.453</v>
       </c>
       <c r="F130" s="5" t="n">
-        <v>0</v>
+        <v>2.56</v>
       </c>
       <c r="G130" s="5" t="n">
-        <v>0</v>
+        <v>0.396</v>
       </c>
       <c r="H130" s="6" t="n">
-        <v>0.2530358</v>
+        <v>0.2489028</v>
       </c>
       <c r="I130" s="6" t="n">
-        <v>0.2530358</v>
+        <v>0.2489028</v>
       </c>
     </row>
     <row r="131">
@@ -4893,16 +4893,16 @@
         <v>1662.656</v>
       </c>
       <c r="F131" s="5" t="n">
-        <v>0</v>
+        <v>2.3</v>
       </c>
       <c r="G131" s="5" t="n">
-        <v>0</v>
+        <v>0.348</v>
       </c>
       <c r="H131" s="6" t="n">
-        <v>0.2095464</v>
+        <v>0.2530358</v>
       </c>
       <c r="I131" s="6" t="n">
-        <v>0.2095464</v>
+        <v>0.2530358</v>
       </c>
     </row>
     <row r="132">
@@ -4924,16 +4924,16 @@
         <v>1662.984</v>
       </c>
       <c r="F132" s="5" t="n">
-        <v>0</v>
+        <v>2.26</v>
       </c>
       <c r="G132" s="5" t="n">
-        <v>0</v>
+        <v>0.313</v>
       </c>
       <c r="H132" s="6" t="n">
-        <v>0.1755135</v>
+        <v>0.2095464</v>
       </c>
       <c r="I132" s="6" t="n">
-        <v>0.1755135</v>
+        <v>0.2095464</v>
       </c>
     </row>
     <row r="133">
@@ -4955,16 +4955,16 @@
         <v>1695.375</v>
       </c>
       <c r="F133" s="5" t="n">
-        <v>0</v>
+        <v>2.09</v>
       </c>
       <c r="G133" s="5" t="n">
-        <v>0</v>
+        <v>0.287</v>
       </c>
       <c r="H133" s="6" t="n">
-        <v>0.2187398</v>
+        <v>0.1755135</v>
       </c>
       <c r="I133" s="6" t="n">
-        <v>0.2187398</v>
+        <v>0.1755135</v>
       </c>
     </row>
     <row r="134">
@@ -4986,16 +4986,16 @@
         <v>1707.328</v>
       </c>
       <c r="F134" s="5" t="n">
-        <v>0</v>
+        <v>1.94</v>
       </c>
       <c r="G134" s="5" t="n">
-        <v>0</v>
+        <v>0.263</v>
       </c>
       <c r="H134" s="6" t="n">
-        <v>0.2640905</v>
+        <v>0.2187398</v>
       </c>
       <c r="I134" s="6" t="n">
-        <v>0.2640905</v>
+        <v>0.2187398</v>
       </c>
     </row>
     <row r="135">
@@ -5017,16 +5017,16 @@
         <v>1723.906</v>
       </c>
       <c r="F135" s="5" t="n">
-        <v>0</v>
+        <v>1.86</v>
       </c>
       <c r="G135" s="5" t="n">
-        <v>0</v>
+        <v>0.245</v>
       </c>
       <c r="H135" s="6" t="n">
-        <v>0.1206024</v>
+        <v>0.2640905</v>
       </c>
       <c r="I135" s="6" t="n">
-        <v>0.1206024</v>
+        <v>0.2640905</v>
       </c>
     </row>
     <row r="136">
@@ -5048,16 +5048,16 @@
         <v>10707.078</v>
       </c>
       <c r="F136" s="5" t="n">
-        <v>0</v>
+        <v>7.91</v>
       </c>
       <c r="G136" s="5" t="n">
-        <v>0</v>
+        <v>1.406</v>
       </c>
       <c r="H136" s="6" t="n">
-        <v>0.1250019</v>
+        <v>0.1206024</v>
       </c>
       <c r="I136" s="6" t="n">
-        <v>0.1250019</v>
+        <v>0.1206024</v>
       </c>
     </row>
     <row r="137">
@@ -5079,16 +5079,16 @@
         <v>11424.781</v>
       </c>
       <c r="F137" s="5" t="n">
-        <v>0</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="G137" s="5" t="n">
-        <v>0</v>
+        <v>1.396</v>
       </c>
       <c r="H137" s="6" t="n">
-        <v>0.2844053</v>
+        <v>0.1250019</v>
       </c>
       <c r="I137" s="6" t="n">
-        <v>0.2844053</v>
+        <v>0.1250019</v>
       </c>
     </row>
     <row r="138">
@@ -5110,16 +5110,16 @@
         <v>11424.781</v>
       </c>
       <c r="F138" s="5" t="n">
-        <v>0</v>
+        <v>7.58</v>
       </c>
       <c r="G138" s="5" t="n">
-        <v>0</v>
+        <v>1.31</v>
       </c>
       <c r="H138" s="6" t="n">
-        <v>0.1176871</v>
+        <v>0.2844053</v>
       </c>
       <c r="I138" s="6" t="n">
-        <v>0.1176871</v>
+        <v>0.2844053</v>
       </c>
     </row>
     <row r="139">
@@ -5141,16 +5141,16 @@
         <v>18184.078</v>
       </c>
       <c r="F139" s="5" t="n">
-        <v>0</v>
+        <v>12.58</v>
       </c>
       <c r="G139" s="5" t="n">
-        <v>0</v>
+        <v>1.95</v>
       </c>
       <c r="H139" s="6" t="n">
-        <v>0.2055215</v>
+        <v>0.1176871</v>
       </c>
       <c r="I139" s="6" t="n">
-        <v>0.2055215</v>
+        <v>0.1176871</v>
       </c>
     </row>
     <row r="140">
@@ -5172,16 +5172,16 @@
         <v>18184.078</v>
       </c>
       <c r="F140" s="5" t="n">
-        <v>0</v>
+        <v>11.88</v>
       </c>
       <c r="G140" s="5" t="n">
-        <v>0</v>
+        <v>1.838</v>
       </c>
       <c r="H140" s="6" t="n">
-        <v>0.1249024</v>
+        <v>0.2055215</v>
       </c>
       <c r="I140" s="6" t="n">
-        <v>0.1249024</v>
+        <v>0.2055215</v>
       </c>
     </row>
     <row r="141">
@@ -5203,16 +5203,16 @@
         <v>26878.344</v>
       </c>
       <c r="F141" s="5" t="n">
-        <v>0</v>
+        <v>15.84</v>
       </c>
       <c r="G141" s="5" t="n">
-        <v>0</v>
+        <v>2.572</v>
       </c>
       <c r="H141" s="6" t="n">
-        <v>0.12151</v>
+        <v>0.1249024</v>
       </c>
       <c r="I141" s="6" t="n">
-        <v>0.12151</v>
+        <v>0.1249024</v>
       </c>
     </row>
     <row r="142">
@@ -5234,16 +5234,16 @@
         <v>31095.625</v>
       </c>
       <c r="F142" s="5" t="n">
-        <v>0</v>
+        <v>17.92</v>
       </c>
       <c r="G142" s="5" t="n">
-        <v>0</v>
+        <v>2.817</v>
       </c>
       <c r="H142" s="6" t="n">
-        <v>0.1979822</v>
+        <v>0.12151</v>
       </c>
       <c r="I142" s="6" t="n">
-        <v>0.1979822</v>
+        <v>0.12151</v>
       </c>
     </row>
     <row r="143">
@@ -5265,16 +5265,16 @@
         <v>31122.781</v>
       </c>
       <c r="F143" s="5" t="n">
-        <v>0</v>
+        <v>17.15</v>
       </c>
       <c r="G143" s="5" t="n">
-        <v>0</v>
+        <v>2.678</v>
       </c>
       <c r="H143" s="6" t="n">
-        <v>0.223656</v>
+        <v>0.1979822</v>
       </c>
       <c r="I143" s="6" t="n">
-        <v>0.223656</v>
+        <v>0.1979822</v>
       </c>
     </row>
     <row r="144">
@@ -5296,16 +5296,16 @@
         <v>31144.969</v>
       </c>
       <c r="F144" s="5" t="n">
-        <v>0</v>
+        <v>16.44</v>
       </c>
       <c r="G144" s="5" t="n">
-        <v>0</v>
+        <v>2.557</v>
       </c>
       <c r="H144" s="6" t="n">
-        <v>0.16747</v>
+        <v>0.223656</v>
       </c>
       <c r="I144" s="6" t="n">
-        <v>0.16747</v>
+        <v>0.223656</v>
       </c>
     </row>
     <row r="145">
@@ -5327,16 +5327,16 @@
         <v>31145.297</v>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0</v>
+        <v>15.76</v>
       </c>
       <c r="G145" s="5" t="n">
-        <v>0</v>
+        <v>2.449</v>
       </c>
       <c r="H145" s="6" t="n">
-        <v>0.2373027</v>
+        <v>0.16747</v>
       </c>
       <c r="I145" s="6" t="n">
-        <v>0.2373027</v>
+        <v>0.16747</v>
       </c>
     </row>
     <row r="146">
@@ -5358,16 +5358,16 @@
         <v>31234.766</v>
       </c>
       <c r="F146" s="5" t="n">
-        <v>0</v>
+        <v>15.22</v>
       </c>
       <c r="G146" s="5" t="n">
-        <v>0</v>
+        <v>2.353</v>
       </c>
       <c r="H146" s="6" t="n">
-        <v>0.2300347</v>
+        <v>0.2373027</v>
       </c>
       <c r="I146" s="6" t="n">
-        <v>0.2300347</v>
+        <v>0.2373027</v>
       </c>
     </row>
     <row r="147">
@@ -5389,16 +5389,16 @@
         <v>31263.094</v>
       </c>
       <c r="F147" s="5" t="n">
-        <v>0</v>
+        <v>14.67</v>
       </c>
       <c r="G147" s="5" t="n">
-        <v>0</v>
+        <v>2.264</v>
       </c>
       <c r="H147" s="6" t="n">
-        <v>0.2614626</v>
+        <v>0.2300347</v>
       </c>
       <c r="I147" s="6" t="n">
-        <v>0.2614626</v>
+        <v>0.2300347</v>
       </c>
     </row>
     <row r="148">
@@ -5420,16 +5420,16 @@
         <v>31269.875</v>
       </c>
       <c r="F148" s="5" t="n">
-        <v>0</v>
+        <v>14.09</v>
       </c>
       <c r="G148" s="5" t="n">
-        <v>0</v>
+        <v>2.171</v>
       </c>
       <c r="H148" s="6" t="n">
-        <v>0.12151</v>
+        <v>0.2614626</v>
       </c>
       <c r="I148" s="6" t="n">
-        <v>0.12151</v>
+        <v>0.2614626</v>
       </c>
     </row>
     <row r="149">
@@ -5451,16 +5451,16 @@
         <v>37437.781</v>
       </c>
       <c r="F149" s="5" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="G149" s="5" t="n">
-        <v>0</v>
+        <v>2.505</v>
       </c>
       <c r="H149" s="6" t="n">
-        <v>0.2501633</v>
+        <v>0.12151</v>
       </c>
       <c r="I149" s="6" t="n">
-        <v>0.2501633</v>
+        <v>0.12151</v>
       </c>
     </row>
     <row r="150">
@@ -5482,16 +5482,16 @@
         <v>37439.125</v>
       </c>
       <c r="F150" s="5" t="n">
-        <v>0</v>
+        <v>16.41</v>
       </c>
       <c r="G150" s="5" t="n">
-        <v>0</v>
+        <v>2.409</v>
       </c>
       <c r="H150" s="6" t="n">
-        <v>0.2537298</v>
+        <v>0.2501633</v>
       </c>
       <c r="I150" s="6" t="n">
-        <v>0.2537298</v>
+        <v>0.2501633</v>
       </c>
     </row>
     <row r="151">
@@ -5513,16 +5513,16 @@
         <v>37459.891</v>
       </c>
       <c r="F151" s="5" t="n">
-        <v>0</v>
+        <v>15.86</v>
       </c>
       <c r="G151" s="5" t="n">
-        <v>0</v>
+        <v>2.325</v>
       </c>
       <c r="H151" s="6" t="n">
-        <v>0.1260111</v>
+        <v>0.2537298</v>
       </c>
       <c r="I151" s="6" t="n">
-        <v>0.1260111</v>
+        <v>0.2537298</v>
       </c>
     </row>
     <row r="152">
@@ -5544,16 +5544,16 @@
         <v>37477.516</v>
       </c>
       <c r="F152" s="5" t="n">
-        <v>0</v>
+        <v>15.32</v>
       </c>
       <c r="G152" s="5" t="n">
-        <v>0</v>
+        <v>2.245</v>
       </c>
       <c r="H152" s="6" t="n">
-        <v>0.1950825</v>
+        <v>0.1260111</v>
       </c>
       <c r="I152" s="6" t="n">
-        <v>0.1950825</v>
+        <v>0.1260111</v>
       </c>
     </row>
     <row r="153">
@@ -5575,16 +5575,16 @@
         <v>37477.516</v>
       </c>
       <c r="F153" s="5" t="n">
-        <v>0</v>
+        <v>14.82</v>
       </c>
       <c r="G153" s="5" t="n">
-        <v>0</v>
+        <v>2.17</v>
       </c>
       <c r="H153" s="6" t="n">
-        <v>0</v>
+        <v>0.1950825</v>
       </c>
       <c r="I153" s="6" t="n">
-        <v>0</v>
+        <v>0.1950825</v>
       </c>
     </row>
     <row r="154">
@@ -5606,16 +5606,16 @@
         <v>6431.938</v>
       </c>
       <c r="F154" s="5" t="n">
-        <v>0</v>
+        <v>40.78</v>
       </c>
       <c r="G154" s="5" t="n">
-        <v>0</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="H154" s="6" t="n">
-        <v>0.1833829</v>
+        <v>0.2557159</v>
       </c>
       <c r="I154" s="6" t="n">
-        <v>0.1833829</v>
+        <v>0.2557159</v>
       </c>
     </row>
     <row r="155">
@@ -5637,16 +5637,16 @@
         <v>6450.078</v>
       </c>
       <c r="F155" s="5" t="n">
-        <v>0</v>
+        <v>21.84</v>
       </c>
       <c r="G155" s="5" t="n">
-        <v>0</v>
+        <v>4.977</v>
       </c>
       <c r="H155" s="6" t="n">
-        <v>0.1209789</v>
+        <v>0.1833829</v>
       </c>
       <c r="I155" s="6" t="n">
-        <v>0.1209789</v>
+        <v>0.1833829</v>
       </c>
     </row>
     <row r="156">
@@ -5668,16 +5668,16 @@
         <v>18357.672</v>
       </c>
       <c r="F156" s="5" t="n">
-        <v>0</v>
+        <v>44.67</v>
       </c>
       <c r="G156" s="5" t="n">
-        <v>0</v>
+        <v>10.148</v>
       </c>
       <c r="H156" s="6" t="n">
-        <v>0.2206865</v>
+        <v>0.1209789</v>
       </c>
       <c r="I156" s="6" t="n">
-        <v>0.2206865</v>
+        <v>0.1209789</v>
       </c>
     </row>
     <row r="157">
@@ -5699,16 +5699,16 @@
         <v>18367.469</v>
       </c>
       <c r="F157" s="5" t="n">
-        <v>0</v>
+        <v>34.23</v>
       </c>
       <c r="G157" s="5" t="n">
-        <v>0</v>
+        <v>7.77</v>
       </c>
       <c r="H157" s="6" t="n">
-        <v>0.2277191</v>
+        <v>0.2206865</v>
       </c>
       <c r="I157" s="6" t="n">
-        <v>0.2277191</v>
+        <v>0.2206865</v>
       </c>
     </row>
     <row r="158">
@@ -5730,16 +5730,16 @@
         <v>18367.625</v>
       </c>
       <c r="F158" s="5" t="n">
-        <v>0</v>
+        <v>27.93</v>
       </c>
       <c r="G158" s="5" t="n">
-        <v>0</v>
+        <v>6.318</v>
       </c>
       <c r="H158" s="6" t="n">
-        <v>0.2844053</v>
+        <v>0.2277191</v>
       </c>
       <c r="I158" s="6" t="n">
-        <v>0.2844053</v>
+        <v>0.2277191</v>
       </c>
     </row>
     <row r="159">
@@ -5761,16 +5761,16 @@
         <v>18456.672</v>
       </c>
       <c r="F159" s="5" t="n">
-        <v>0</v>
+        <v>24.95</v>
       </c>
       <c r="G159" s="5" t="n">
-        <v>0</v>
+        <v>5.13</v>
       </c>
       <c r="H159" s="6" t="n">
-        <v>0.2265649</v>
+        <v>0.2844053</v>
       </c>
       <c r="I159" s="6" t="n">
-        <v>0.2265649</v>
+        <v>0.2844053</v>
       </c>
     </row>
     <row r="160">
@@ -5792,16 +5792,16 @@
         <v>23778.219</v>
       </c>
       <c r="F160" s="5" t="n">
-        <v>0</v>
+        <v>28.21</v>
       </c>
       <c r="G160" s="5" t="n">
-        <v>0</v>
+        <v>5.726</v>
       </c>
       <c r="H160" s="6" t="n">
-        <v>0.1260111</v>
+        <v>0.2265649</v>
       </c>
       <c r="I160" s="6" t="n">
-        <v>0.1260111</v>
+        <v>0.2265649</v>
       </c>
     </row>
     <row r="161">
@@ -5823,16 +5823,16 @@
         <v>24339.938</v>
       </c>
       <c r="F161" s="5" t="n">
-        <v>0</v>
+        <v>25.29</v>
       </c>
       <c r="G161" s="5" t="n">
-        <v>0</v>
+        <v>5.135</v>
       </c>
       <c r="H161" s="6" t="n">
-        <v>0.2316885</v>
+        <v>0.1260111</v>
       </c>
       <c r="I161" s="6" t="n">
-        <v>0.2316885</v>
+        <v>0.1260111</v>
       </c>
     </row>
     <row r="162">
@@ -5854,16 +5854,16 @@
         <v>24339.938</v>
       </c>
       <c r="F162" s="5" t="n">
-        <v>0</v>
+        <v>22.79</v>
       </c>
       <c r="G162" s="5" t="n">
-        <v>0</v>
+        <v>4.614</v>
       </c>
       <c r="H162" s="6" t="n">
-        <v>0.294502</v>
+        <v>0.2316885</v>
       </c>
       <c r="I162" s="6" t="n">
-        <v>0.294502</v>
+        <v>0.2316885</v>
       </c>
     </row>
     <row r="163">
@@ -5885,16 +5885,16 @@
         <v>24492.313</v>
       </c>
       <c r="F163" s="5" t="n">
-        <v>0</v>
+        <v>23.78</v>
       </c>
       <c r="G163" s="5" t="n">
-        <v>0</v>
+        <v>4.178</v>
       </c>
       <c r="H163" s="6" t="n">
-        <v>0.12151</v>
+        <v>0.294502</v>
       </c>
       <c r="I163" s="6" t="n">
-        <v>0.12151</v>
+        <v>0.294502</v>
       </c>
     </row>
     <row r="164">
@@ -5916,16 +5916,16 @@
         <v>32919.969</v>
       </c>
       <c r="F164" s="5" t="n">
-        <v>0</v>
+        <v>28.24</v>
       </c>
       <c r="G164" s="5" t="n">
-        <v>0</v>
+        <v>5.133</v>
       </c>
       <c r="H164" s="6" t="n">
-        <v>0.1822086</v>
+        <v>0.12151</v>
       </c>
       <c r="I164" s="6" t="n">
-        <v>0.1822086</v>
+        <v>0.12151</v>
       </c>
     </row>
     <row r="165">
@@ -5947,16 +5947,16 @@
         <v>33243.281</v>
       </c>
       <c r="F165" s="5" t="n">
-        <v>0</v>
+        <v>26.32</v>
       </c>
       <c r="G165" s="5" t="n">
-        <v>0</v>
+        <v>4.757</v>
       </c>
       <c r="H165" s="6" t="n">
-        <v>0.2793801</v>
+        <v>0.1822086</v>
       </c>
       <c r="I165" s="6" t="n">
-        <v>0.2793801</v>
+        <v>0.1822086</v>
       </c>
     </row>
     <row r="166">
@@ -5978,16 +5978,16 @@
         <v>33252.563</v>
       </c>
       <c r="F166" s="5" t="n">
-        <v>0</v>
+        <v>27.18</v>
       </c>
       <c r="G166" s="5" t="n">
-        <v>0</v>
+        <v>4.383</v>
       </c>
       <c r="H166" s="6" t="n">
-        <v>0.1252291</v>
+        <v>0.2793801</v>
       </c>
       <c r="I166" s="6" t="n">
-        <v>0.1252291</v>
+        <v>0.2793801</v>
       </c>
     </row>
     <row r="167">
@@ -6009,16 +6009,16 @@
         <v>33265.25</v>
       </c>
       <c r="F167" s="5" t="n">
-        <v>0</v>
+        <v>25.29</v>
       </c>
       <c r="G167" s="5" t="n">
-        <v>0</v>
+        <v>4.074</v>
       </c>
       <c r="H167" s="6" t="n">
-        <v>0.1904234</v>
+        <v>0.1252291</v>
       </c>
       <c r="I167" s="6" t="n">
-        <v>0.1904234</v>
+        <v>0.1252291</v>
       </c>
     </row>
     <row r="168">
@@ -6040,16 +6040,16 @@
         <v>33293.609</v>
       </c>
       <c r="F168" s="5" t="n">
-        <v>0</v>
+        <v>23.62</v>
       </c>
       <c r="G168" s="5" t="n">
-        <v>0</v>
+        <v>3.802</v>
       </c>
       <c r="H168" s="6" t="n">
-        <v>0.2459873</v>
+        <v>0.1904234</v>
       </c>
       <c r="I168" s="6" t="n">
-        <v>0.2459873</v>
+        <v>0.1904234</v>
       </c>
     </row>
     <row r="169">
@@ -6071,16 +6071,16 @@
         <v>33333.141</v>
       </c>
       <c r="F169" s="5" t="n">
-        <v>0</v>
+        <v>22.22</v>
       </c>
       <c r="G169" s="5" t="n">
-        <v>0</v>
+        <v>3.575</v>
       </c>
       <c r="H169" s="6" t="n">
-        <v>0.2452898</v>
+        <v>0.2459873</v>
       </c>
       <c r="I169" s="6" t="n">
-        <v>0.2452898</v>
+        <v>0.2459873</v>
       </c>
     </row>
     <row r="170">
@@ -6102,16 +6102,16 @@
         <v>33368.719</v>
       </c>
       <c r="F170" s="5" t="n">
-        <v>0</v>
+        <v>20.81</v>
       </c>
       <c r="G170" s="5" t="n">
-        <v>0</v>
+        <v>3.347</v>
       </c>
       <c r="H170" s="6" t="n">
-        <v>0.1234443</v>
+        <v>0.2452898</v>
       </c>
       <c r="I170" s="6" t="n">
-        <v>0.1234443</v>
+        <v>0.2452898</v>
       </c>
     </row>
     <row r="171">
@@ -6133,16 +6133,16 @@
         <v>38083.016</v>
       </c>
       <c r="F171" s="5" t="n">
-        <v>0</v>
+        <v>21.42</v>
       </c>
       <c r="G171" s="5" t="n">
-        <v>0</v>
+        <v>3.596</v>
       </c>
       <c r="H171" s="6" t="n">
-        <v>0.2363978</v>
+        <v>0.1234443</v>
       </c>
       <c r="I171" s="6" t="n">
-        <v>0.2363978</v>
+        <v>0.1234443</v>
       </c>
     </row>
     <row r="172">
@@ -6164,16 +6164,16 @@
         <v>38083.875</v>
       </c>
       <c r="F172" s="5" t="n">
-        <v>0</v>
+        <v>20.28</v>
       </c>
       <c r="G172" s="5" t="n">
-        <v>0</v>
+        <v>3.402</v>
       </c>
       <c r="H172" s="6" t="n">
-        <v>0.269941</v>
+        <v>0.2363978</v>
       </c>
       <c r="I172" s="6" t="n">
-        <v>0.269941</v>
+        <v>0.2363978</v>
       </c>
     </row>
     <row r="173">
@@ -6195,16 +6195,16 @@
         <v>38105.266</v>
       </c>
       <c r="F173" s="5" t="n">
-        <v>0</v>
+        <v>19.25</v>
       </c>
       <c r="G173" s="5" t="n">
-        <v>0</v>
+        <v>3.222</v>
       </c>
       <c r="H173" s="6" t="n">
-        <v>0.2643565</v>
+        <v>0.269941</v>
       </c>
       <c r="I173" s="6" t="n">
-        <v>0.2643565</v>
+        <v>0.269941</v>
       </c>
     </row>
     <row r="174">
@@ -6226,16 +6226,16 @@
         <v>38124.609</v>
       </c>
       <c r="F174" s="5" t="n">
-        <v>0</v>
+        <v>18.45</v>
       </c>
       <c r="G174" s="5" t="n">
-        <v>0</v>
+        <v>3.082</v>
       </c>
       <c r="H174" s="6" t="n">
-        <v>0.1202812</v>
+        <v>0.2643565</v>
       </c>
       <c r="I174" s="6" t="n">
-        <v>0.1202812</v>
+        <v>0.2643565</v>
       </c>
     </row>
     <row r="175">
@@ -6257,16 +6257,16 @@
         <v>50405.875</v>
       </c>
       <c r="F175" s="5" t="n">
-        <v>0</v>
+        <v>21.65</v>
       </c>
       <c r="G175" s="5" t="n">
-        <v>0</v>
+        <v>3.908</v>
       </c>
       <c r="H175" s="6" t="n">
-        <v>0.2222444</v>
+        <v>0.1202812</v>
       </c>
       <c r="I175" s="6" t="n">
-        <v>0.2222444</v>
+        <v>0.1202812</v>
       </c>
     </row>
     <row r="176">
@@ -6288,16 +6288,16 @@
         <v>51554.469</v>
       </c>
       <c r="F176" s="5" t="n">
-        <v>0</v>
+        <v>21.17</v>
       </c>
       <c r="G176" s="5" t="n">
-        <v>0</v>
+        <v>3.837</v>
       </c>
       <c r="H176" s="6" t="n">
-        <v>0.193604</v>
+        <v>0.2222444</v>
       </c>
       <c r="I176" s="6" t="n">
-        <v>0.193604</v>
+        <v>0.2222444</v>
       </c>
     </row>
     <row r="177">
@@ -6319,16 +6319,16 @@
         <v>51562.969</v>
       </c>
       <c r="F177" s="5" t="n">
-        <v>0</v>
+        <v>20.33</v>
       </c>
       <c r="G177" s="5" t="n">
-        <v>0</v>
+        <v>3.682</v>
       </c>
       <c r="H177" s="6" t="n">
-        <v>0.2632921</v>
+        <v>0.193604</v>
       </c>
       <c r="I177" s="6" t="n">
-        <v>0.2632921</v>
+        <v>0.193604</v>
       </c>
     </row>
     <row r="178">
@@ -6350,16 +6350,16 @@
         <v>51571.891</v>
       </c>
       <c r="F178" s="5" t="n">
-        <v>0</v>
+        <v>19.61</v>
       </c>
       <c r="G178" s="5" t="n">
-        <v>0</v>
+        <v>3.549</v>
       </c>
       <c r="H178" s="6" t="n">
-        <v>0.1840018</v>
+        <v>0.2632921</v>
       </c>
       <c r="I178" s="6" t="n">
-        <v>0.1840018</v>
+        <v>0.2632921</v>
       </c>
     </row>
     <row r="179">
@@ -6381,16 +6381,16 @@
         <v>51596.906</v>
       </c>
       <c r="F179" s="5" t="n">
-        <v>0</v>
+        <v>18.84</v>
       </c>
       <c r="G179" s="5" t="n">
-        <v>0</v>
+        <v>3.406</v>
       </c>
       <c r="H179" s="6" t="n">
-        <v>0.2916649</v>
+        <v>0.1840018</v>
       </c>
       <c r="I179" s="6" t="n">
-        <v>0.2916649</v>
+        <v>0.1840018</v>
       </c>
     </row>
     <row r="180">
@@ -6412,16 +6412,16 @@
         <v>57935.375</v>
       </c>
       <c r="F180" s="5" t="n">
-        <v>0</v>
+        <v>20.24</v>
       </c>
       <c r="G180" s="5" t="n">
-        <v>0</v>
+        <v>3.674</v>
       </c>
       <c r="H180" s="6" t="n">
-        <v>0.2448948</v>
+        <v>0.2916649</v>
       </c>
       <c r="I180" s="6" t="n">
-        <v>0.2448948</v>
+        <v>0.2916649</v>
       </c>
     </row>
     <row r="181">
@@ -6443,16 +6443,16 @@
         <v>57944.328</v>
       </c>
       <c r="F181" s="5" t="n">
-        <v>0</v>
+        <v>19.47</v>
       </c>
       <c r="G181" s="5" t="n">
-        <v>0</v>
+        <v>3.528</v>
       </c>
       <c r="H181" s="6" t="n">
-        <v>0.2639391</v>
+        <v>0.2448948</v>
       </c>
       <c r="I181" s="6" t="n">
-        <v>0.2639391</v>
+        <v>0.2448948</v>
       </c>
     </row>
     <row r="182">
@@ -6474,16 +6474,16 @@
         <v>57945.172</v>
       </c>
       <c r="F182" s="5" t="n">
-        <v>0</v>
+        <v>18.8</v>
       </c>
       <c r="G182" s="5" t="n">
-        <v>0</v>
+        <v>3.402</v>
       </c>
       <c r="H182" s="6" t="n">
-        <v>0.2024876</v>
+        <v>0.2639391</v>
       </c>
       <c r="I182" s="6" t="n">
-        <v>0.2024876</v>
+        <v>0.2639391</v>
       </c>
     </row>
     <row r="183">
@@ -6505,16 +6505,16 @@
         <v>57986.563</v>
       </c>
       <c r="F183" s="5" t="n">
-        <v>0</v>
+        <v>18.21</v>
       </c>
       <c r="G183" s="5" t="n">
-        <v>0</v>
+        <v>3.288</v>
       </c>
       <c r="H183" s="6" t="n">
-        <v>0</v>
+        <v>0.2024876</v>
       </c>
       <c r="I183" s="6" t="n">
-        <v>0</v>
+        <v>0.2024876</v>
       </c>
     </row>
   </sheetData>

</xml_diff>